<commit_message>
PediDoses v0.9 : corriger le protocole SMUR et préparer les réglages de posologie
Appliquer les corrections de doses, plafonds, ampoules, voies et dilutions du 26 septembre 2026. Conserver le sufentanil en mcg (50 mcg/10 mL). Ajouter Propofol LISA, la deuxième dose de triphosadénine et la charge de nicardipine.

Ajouter les commandes +/− aux 14 perfusions continues et à la charge de nicardipine, avec recalcul à concentration constante. Les pas restent à définir par l’utilisateur ; les commandes sont désactivées en attendant. Ne pas inventer la dilution du gluconate ni la concentration d’entretien de tranexamique avant 10 ans.

Actualiser le classeur de 66 ampoules et la documentation. Vérification syntaxique et 67 tests réussis. Rendu de l’application non vérifié : accès du navigateur au serveur local bloqué.
</commit_message>
<xml_diff>
--- a/dist/assets/PediDoses-Ampoules.xlsx
+++ b/dist/assets/PediDoses-Ampoules.xlsx
@@ -2,8 +2,8 @@
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <x:workbook xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <x:sheets>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Ampoules" sheetId="1" r:id="Rf57250932de44da1"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Mode d’emploi" sheetId="2" r:id="R8f02eb54d57f454b"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Ampoules" sheetId="1" r:id="Rd80d76bd82294721"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Mode d’emploi" sheetId="2" r:id="Raf2bd21fd0034aa6"/>
   </x:sheets>
 </x:workbook>
 </file>
@@ -14,10 +14,11 @@
 
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
 <x:styleSheet xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
-  <x:numFmts count="1">
+  <x:numFmts count="2">
     <x:numFmt numFmtId="200" formatCode="0.00##########"/>
+    <x:numFmt numFmtId="201" formatCode="0.00"/>
   </x:numFmts>
-  <x:fonts count="4">
+  <x:fonts count="5">
     <x:font>
       <x:sz val="11"/>
       <x:name val="Carlito"/>
@@ -37,8 +38,12 @@
       <x:sz val="11"/>
       <x:name val="Arial"/>
     </x:font>
+    <x:font>
+      <x:sz val="10"/>
+      <x:name val="Arial"/>
+    </x:font>
   </x:fonts>
-  <x:fills count="5">
+  <x:fills count="7">
     <x:fill>
       <x:patternFill patternType="none"/>
     </x:fill>
@@ -60,6 +65,16 @@
         <x:fgColor rgb="FFF2F4F6"/>
       </x:patternFill>
     </x:fill>
+    <x:fill>
+      <x:patternFill patternType="solid">
+        <x:fgColor rgb="FFFFF2CC"/>
+      </x:patternFill>
+    </x:fill>
+    <x:fill>
+      <x:patternFill patternType="solid">
+        <x:fgColor rgb="FFE7E6E6"/>
+      </x:patternFill>
+    </x:fill>
   </x:fills>
   <x:borders count="2">
     <x:border/>
@@ -72,7 +87,7 @@
   <x:cellStyleXfs count="1">
     <x:xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </x:cellStyleXfs>
-  <x:cellXfs count="16">
+  <x:cellXfs count="23">
     <x:xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <x:xf numFmtId="0" fontId="1" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1"/>
     <x:xf numFmtId="0" fontId="1" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
@@ -117,6 +132,25 @@
     <x:xf numFmtId="0" fontId="3" fillId="2" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <x:alignment vertical="center" wrapText="1"/>
     </x:xf>
+    <x:xf numFmtId="0" fontId="4" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1"/>
+    <x:xf numFmtId="0" fontId="4" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <x:alignment wrapText="1"/>
+    </x:xf>
+    <x:xf numFmtId="0" fontId="4" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <x:alignment vertical="center" wrapText="1"/>
+    </x:xf>
+    <x:xf numFmtId="0" fontId="4" fillId="5" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <x:alignment vertical="center" wrapText="1"/>
+    </x:xf>
+    <x:xf numFmtId="0" fontId="4" fillId="6" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <x:alignment vertical="center" wrapText="1"/>
+    </x:xf>
+    <x:xf numFmtId="201" fontId="4" fillId="5" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <x:alignment vertical="center" wrapText="1"/>
+    </x:xf>
+    <x:xf numFmtId="201" fontId="4" fillId="6" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <x:alignment vertical="center" wrapText="1"/>
+    </x:xf>
   </x:cellXfs>
   <x:cellStyles count="1">
     <x:cellStyle name="Normal" xfId="0"/>
@@ -124,7 +158,7 @@
   <x:dxfs count="1">
     <x:dxf>
       <x:fill>
-        <x:patternFill patternType="solid">
+        <x:patternFill>
           <x:bgColor rgb="FFFFF1D6"/>
         </x:patternFill>
       </x:fill>
@@ -134,8 +168,8 @@
 </file>
 
 <file path=xl/tables/table1.xml><?xml version="1.0" encoding="utf-8"?>
-<x:table xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main" id="1" name="AmpoulesPediDoses" displayName="AmpoulesPediDoses" ref="A1:L64" headerRowCount="1" totalsRowCount="0" totalsRowShown="0">
-  <x:autoFilter ref="A1:L64"/>
+<x:table xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main" id="1" name="AmpoulesPediDoses" displayName="AmpoulesPediDoses" ref="A1:L67" headerRowCount="1" totalsRowCount="0" totalsRowShown="0">
+  <x:autoFilter ref="A1:L67"/>
   <x:tableColumns count="12">
     <x:tableColumn id="1" name="Identifiant"/>
     <x:tableColumn id="2" name="Médicament"/>
@@ -516,23 +550,25 @@
       <x:c r="C5" s="3" t="str">
         <x:v>Chlorure de calcium</x:v>
       </x:c>
-      <x:c r="D5" s="7"/>
-      <x:c r="E5" s="7"/>
+      <x:c r="D5" s="7" t="n">
+        <x:v>10</x:v>
+      </x:c>
+      <x:c r="E5" s="7" t="n">
+        <x:v>1000</x:v>
+      </x:c>
       <x:c r="F5" s="6" t="str">
         <x:v>mg</x:v>
       </x:c>
-      <x:c r="G5" s="7" t="n">
-        <x:v>100</x:v>
-      </x:c>
+      <x:c r="G5" s="7"/>
       <x:c r="H5" s="9" t="n">
         <x:f>IF(AND(ISNUMBER(D5),D5&gt;0,ISNUMBER(E5),E5&gt;0),E5/D5,IF(ISNUMBER(G5),G5,""))</x:f>
         <x:v>100</x:v>
       </x:c>
       <x:c r="I5" s="3" t="str">
-        <x:v>chlorure de calcium — expression de dose à confirmer</x:v>
+        <x:v>chlorure de calcium</x:v>
       </x:c>
       <x:c r="J5" s="3" t="str">
-        <x:v>à confirmer</x:v>
+        <x:v>confirmé</x:v>
       </x:c>
       <x:c r="K5" s="3" t="str"/>
       <x:c r="L5" s="3" t="str">
@@ -670,10 +706,12 @@
         <x:v>Amoxicilline / acide clavulanique</x:v>
       </x:c>
       <x:c r="C10" s="3" t="str">
-        <x:v>Poudre pour solution injectable</x:v>
+        <x:v>Poudre pour solution injectable 500 mg/50 mg</x:v>
       </x:c>
       <x:c r="D10" s="7"/>
-      <x:c r="E10" s="7"/>
+      <x:c r="E10" s="7" t="n">
+        <x:v>500</x:v>
+      </x:c>
       <x:c r="F10" s="6" t="str">
         <x:v>mg</x:v>
       </x:c>
@@ -682,14 +720,12 @@
         <x:f>IF(AND(ISNUMBER(D10),D10&gt;0,ISNUMBER(E10),E10&gt;0),E10/D10,IF(ISNUMBER(G10),G10,""))</x:f>
       </x:c>
       <x:c r="I10" s="3" t="str">
-        <x:v>amoxicilline</x:v>
+        <x:v>amoxicilline (500 mg / 50 mg d’acide clavulanique)</x:v>
       </x:c>
       <x:c r="J10" s="3" t="str">
-        <x:v>à confirmer</x:v>
-      </x:c>
-      <x:c r="K10" s="3" t="str">
-        <x:v>Renseigner le dosage et le rapport amoxicilline/acide clavulanique.</x:v>
-      </x:c>
+        <x:v>confirmé</x:v>
+      </x:c>
+      <x:c r="K10" s="3" t="str"/>
       <x:c r="L10" s="3" t="str">
         <x:v>Tableau Prescription / Ampoules et décisions locales de la conversation</x:v>
       </x:c>
@@ -871,28 +907,29 @@
         <x:v>Sulfate de magnésium</x:v>
       </x:c>
       <x:c r="C16" s="3" t="str">
-        <x:v>Sulfate magnéisum</x:v>
+        <x:v>Sulfate de magnésium 15 %</x:v>
       </x:c>
       <x:c r="D16" s="7" t="n">
         <x:v>10</x:v>
       </x:c>
-      <x:c r="E16" s="7"/>
+      <x:c r="E16" s="7" t="n">
+        <x:v>1.5</x:v>
+      </x:c>
       <x:c r="F16" s="6" t="str">
         <x:v>g</x:v>
       </x:c>
       <x:c r="G16" s="7"/>
-      <x:c r="H16" s="9" t="str">
+      <x:c r="H16" s="9" t="n">
         <x:f>IF(AND(ISNUMBER(D16),D16&gt;0,ISNUMBER(E16),E16&gt;0),E16/D16,IF(ISNUMBER(G16),G16,""))</x:f>
+        <x:v>0.15</x:v>
       </x:c>
       <x:c r="I16" s="3" t="str">
         <x:v>sulfate de magnésium</x:v>
       </x:c>
       <x:c r="J16" s="3" t="str">
-        <x:v>à confirmer</x:v>
-      </x:c>
-      <x:c r="K16" s="3" t="str">
-        <x:v>À trancher : 0,15 g par mL (= 1,5 g/10 mL à 15 %) ou 0,15 g par ampoule de 10 mL. Quantité volontairement vide.</x:v>
-      </x:c>
+        <x:v>confirmé</x:v>
+      </x:c>
+      <x:c r="K16" s="3" t="str"/>
       <x:c r="L16" s="3" t="str">
         <x:v>https://base-donnees-publique.medicaments.gouv.fr/medicament/61106121/extrait</x:v>
       </x:c>
@@ -902,7 +939,7 @@
         <x:v>triphosadenine</x:v>
       </x:c>
       <x:c r="B17" s="3" t="str">
-        <x:v>Triphosadénine</x:v>
+        <x:v>Triphosadénine — 1re dose</x:v>
       </x:c>
       <x:c r="C17" s="3" t="str">
         <x:v>Striadyne</x:v>
@@ -922,7 +959,7 @@
         <x:v>10</x:v>
       </x:c>
       <x:c r="I17" s="3" t="str">
-        <x:v>Triphosadénine</x:v>
+        <x:v>Triphosadénine — 1re dose</x:v>
       </x:c>
       <x:c r="J17" s="3" t="str">
         <x:v>à confirmer</x:v>
@@ -1135,7 +1172,7 @@
         <x:v>Morphine (titration)</x:v>
       </x:c>
       <x:c r="J23" s="3" t="str">
-        <x:v>à confirmer</x:v>
+        <x:v>confirmé</x:v>
       </x:c>
       <x:c r="K23" s="3" t="str"/>
       <x:c r="L23" s="3" t="str">
@@ -1152,14 +1189,16 @@
       <x:c r="C24" s="3" t="str">
         <x:v>Propofol</x:v>
       </x:c>
-      <x:c r="D24" s="7"/>
-      <x:c r="E24" s="7"/>
+      <x:c r="D24" s="7" t="n">
+        <x:v>20</x:v>
+      </x:c>
+      <x:c r="E24" s="7" t="n">
+        <x:v>200</x:v>
+      </x:c>
       <x:c r="F24" s="6" t="str">
         <x:v>mg</x:v>
       </x:c>
-      <x:c r="G24" s="7" t="n">
-        <x:v>10</x:v>
-      </x:c>
+      <x:c r="G24" s="7"/>
       <x:c r="H24" s="9" t="n">
         <x:f>IF(AND(ISNUMBER(D24),D24&gt;0,ISNUMBER(E24),E24&gt;0),E24/D24,IF(ISNUMBER(G24),G24,""))</x:f>
         <x:v>10</x:v>
@@ -1168,7 +1207,7 @@
         <x:v>Propofol</x:v>
       </x:c>
       <x:c r="J24" s="3" t="str">
-        <x:v>à confirmer</x:v>
+        <x:v>confirmé</x:v>
       </x:c>
       <x:c r="K24" s="3" t="str"/>
       <x:c r="L24" s="3" t="str">
@@ -1180,28 +1219,30 @@
         <x:v>suxamethonium</x:v>
       </x:c>
       <x:c r="B25" s="3" t="str">
-        <x:v>Suxaméthonium</x:v>
+        <x:v>Suxaméthonium (Célocurine)</x:v>
       </x:c>
       <x:c r="C25" s="3" t="str">
-        <x:v>Celocurine</x:v>
-      </x:c>
-      <x:c r="D25" s="7"/>
-      <x:c r="E25" s="7"/>
+        <x:v>Célocurine</x:v>
+      </x:c>
+      <x:c r="D25" s="7" t="n">
+        <x:v>2</x:v>
+      </x:c>
+      <x:c r="E25" s="7" t="n">
+        <x:v>100</x:v>
+      </x:c>
       <x:c r="F25" s="6" t="str">
         <x:v>mg</x:v>
       </x:c>
-      <x:c r="G25" s="7" t="n">
-        <x:v>50</x:v>
-      </x:c>
+      <x:c r="G25" s="7"/>
       <x:c r="H25" s="9" t="n">
         <x:f>IF(AND(ISNUMBER(D25),D25&gt;0,ISNUMBER(E25),E25&gt;0),E25/D25,IF(ISNUMBER(G25),G25,""))</x:f>
         <x:v>50</x:v>
       </x:c>
       <x:c r="I25" s="3" t="str">
-        <x:v>Suxaméthonium</x:v>
+        <x:v>Suxaméthonium (Célocurine)</x:v>
       </x:c>
       <x:c r="J25" s="3" t="str">
-        <x:v>à confirmer</x:v>
+        <x:v>confirmé</x:v>
       </x:c>
       <x:c r="K25" s="3" t="str"/>
       <x:c r="L25" s="3" t="str">
@@ -1251,7 +1292,7 @@
         <x:v>Clonazépam</x:v>
       </x:c>
       <x:c r="C27" s="3" t="str">
-        <x:v>Rivotril</x:v>
+        <x:v>Clonazépam — ampoule seule</x:v>
       </x:c>
       <x:c r="D27" s="7" t="n">
         <x:v>1</x:v>
@@ -1271,7 +1312,7 @@
         <x:v>Clonazépam</x:v>
       </x:c>
       <x:c r="J27" s="3" t="str">
-        <x:v>à confirmer</x:v>
+        <x:v>confirmé</x:v>
       </x:c>
       <x:c r="K27" s="3" t="str"/>
       <x:c r="L27" s="3" t="str">
@@ -1395,14 +1436,16 @@
       <x:c r="C31" s="3" t="str">
         <x:v>Keppra</x:v>
       </x:c>
-      <x:c r="D31" s="7"/>
-      <x:c r="E31" s="7"/>
+      <x:c r="D31" s="7" t="n">
+        <x:v>5</x:v>
+      </x:c>
+      <x:c r="E31" s="7" t="n">
+        <x:v>500</x:v>
+      </x:c>
       <x:c r="F31" s="6" t="str">
         <x:v>mg</x:v>
       </x:c>
-      <x:c r="G31" s="7" t="n">
-        <x:v>100</x:v>
-      </x:c>
+      <x:c r="G31" s="7"/>
       <x:c r="H31" s="9" t="n">
         <x:f>IF(AND(ISNUMBER(D31),D31&gt;0,ISNUMBER(E31),E31&gt;0),E31/D31,IF(ISNUMBER(G31),G31,""))</x:f>
         <x:v>100</x:v>
@@ -1411,7 +1454,7 @@
         <x:v>Lévétiracétam</x:v>
       </x:c>
       <x:c r="J31" s="3" t="str">
-        <x:v>à confirmer</x:v>
+        <x:v>confirmé</x:v>
       </x:c>
       <x:c r="K31" s="3" t="str"/>
       <x:c r="L31" s="3" t="str">
@@ -1479,11 +1522,9 @@
         <x:v>chlorure de sodium</x:v>
       </x:c>
       <x:c r="J33" s="3" t="str">
-        <x:v>à confirmer</x:v>
-      </x:c>
-      <x:c r="K33" s="3" t="str">
-        <x:v>Préparation fournie par la pharmacie ; aucune dilution à réaliser.</x:v>
-      </x:c>
+        <x:v>confirmé</x:v>
+      </x:c>
+      <x:c r="K33" s="3" t="str"/>
       <x:c r="L33" s="3" t="str">
         <x:v>Tableau Prescription / Ampoules et décisions locales de la conversation</x:v>
       </x:c>
@@ -1549,7 +1590,7 @@
         <x:v>citrate de caféine</x:v>
       </x:c>
       <x:c r="J35" s="3" t="str">
-        <x:v>à confirmer</x:v>
+        <x:v>confirmé</x:v>
       </x:c>
       <x:c r="K35" s="3" t="str"/>
       <x:c r="L35" s="3" t="str">
@@ -1566,14 +1607,16 @@
       <x:c r="C36" s="3" t="str">
         <x:v>Flumazenil</x:v>
       </x:c>
-      <x:c r="D36" s="7"/>
-      <x:c r="E36" s="7"/>
+      <x:c r="D36" s="7" t="n">
+        <x:v>10</x:v>
+      </x:c>
+      <x:c r="E36" s="7" t="n">
+        <x:v>1</x:v>
+      </x:c>
       <x:c r="F36" s="6" t="str">
         <x:v>mg</x:v>
       </x:c>
-      <x:c r="G36" s="7" t="n">
-        <x:v>0.1</x:v>
-      </x:c>
+      <x:c r="G36" s="7"/>
       <x:c r="H36" s="9" t="n">
         <x:f>IF(AND(ISNUMBER(D36),D36&gt;0,ISNUMBER(E36),E36&gt;0),E36/D36,IF(ISNUMBER(G36),G36,""))</x:f>
         <x:v>0.1</x:v>
@@ -1582,7 +1625,7 @@
         <x:v>Flumazénil</x:v>
       </x:c>
       <x:c r="J36" s="3" t="str">
-        <x:v>à confirmer</x:v>
+        <x:v>confirmé</x:v>
       </x:c>
       <x:c r="K36" s="3" t="str"/>
       <x:c r="L36" s="3" t="str">
@@ -1599,14 +1642,16 @@
       <x:c r="C37" s="3" t="str">
         <x:v>Bridion</x:v>
       </x:c>
-      <x:c r="D37" s="7"/>
-      <x:c r="E37" s="7"/>
+      <x:c r="D37" s="7" t="n">
+        <x:v>2</x:v>
+      </x:c>
+      <x:c r="E37" s="7" t="n">
+        <x:v>200</x:v>
+      </x:c>
       <x:c r="F37" s="6" t="str">
         <x:v>mg</x:v>
       </x:c>
-      <x:c r="G37" s="7" t="n">
-        <x:v>100</x:v>
-      </x:c>
+      <x:c r="G37" s="7"/>
       <x:c r="H37" s="9" t="n">
         <x:f>IF(AND(ISNUMBER(D37),D37&gt;0,ISNUMBER(E37),E37&gt;0),E37/D37,IF(ISNUMBER(G37),G37,""))</x:f>
         <x:v>100</x:v>
@@ -1615,7 +1660,7 @@
         <x:v>Sugammadex</x:v>
       </x:c>
       <x:c r="J37" s="3" t="str">
-        <x:v>à confirmer</x:v>
+        <x:v>confirmé</x:v>
       </x:c>
       <x:c r="K37" s="3" t="str"/>
       <x:c r="L37" s="3" t="str">
@@ -1648,7 +1693,7 @@
         <x:v>glucose</x:v>
       </x:c>
       <x:c r="J38" s="3" t="str">
-        <x:v>à confirmer</x:v>
+        <x:v>confirmé</x:v>
       </x:c>
       <x:c r="K38" s="3" t="str"/>
       <x:c r="L38" s="3" t="str">
@@ -1665,14 +1710,16 @@
       <x:c r="C39" s="3" t="str">
         <x:v>Naloxone</x:v>
       </x:c>
-      <x:c r="D39" s="7"/>
-      <x:c r="E39" s="7"/>
+      <x:c r="D39" s="7" t="n">
+        <x:v>1</x:v>
+      </x:c>
+      <x:c r="E39" s="7" t="n">
+        <x:v>0.4</x:v>
+      </x:c>
       <x:c r="F39" s="6" t="str">
         <x:v>mg</x:v>
       </x:c>
-      <x:c r="G39" s="7" t="n">
-        <x:v>0.4</x:v>
-      </x:c>
+      <x:c r="G39" s="7"/>
       <x:c r="H39" s="9" t="n">
         <x:f>IF(AND(ISNUMBER(D39),D39&gt;0,ISNUMBER(E39),E39&gt;0),E39/D39,IF(ISNUMBER(G39),G39,""))</x:f>
         <x:v>0.4</x:v>
@@ -1681,7 +1728,7 @@
         <x:v>Naloxone</x:v>
       </x:c>
       <x:c r="J39" s="3" t="str">
-        <x:v>à confirmer</x:v>
+        <x:v>confirmé</x:v>
       </x:c>
       <x:c r="K39" s="3" t="str"/>
       <x:c r="L39" s="3" t="str">
@@ -1823,7 +1870,9 @@
       <x:c r="J43" s="3" t="str">
         <x:v>à confirmer</x:v>
       </x:c>
-      <x:c r="K43" s="3" t="str"/>
+      <x:c r="K43" s="3" t="str">
+        <x:v>Confirmer le conditionnement disponible ; la cible de préparation est 1 mg/mL.</x:v>
+      </x:c>
       <x:c r="L43" s="3" t="str">
         <x:v>Tableau Prescription / Ampoules et décisions locales de la conversation</x:v>
       </x:c>
@@ -1836,7 +1885,7 @@
         <x:v>Clonazépam (IVSE)</x:v>
       </x:c>
       <x:c r="C44" s="3" t="str">
-        <x:v>Rivotril</x:v>
+        <x:v>Clonazépam — ampoule seule</x:v>
       </x:c>
       <x:c r="D44" s="7" t="n">
         <x:v>1</x:v>
@@ -1856,7 +1905,7 @@
         <x:v>Clonazépam</x:v>
       </x:c>
       <x:c r="J44" s="3" t="str">
-        <x:v>à confirmer</x:v>
+        <x:v>confirmé</x:v>
       </x:c>
       <x:c r="K44" s="3" t="str"/>
       <x:c r="L44" s="3" t="str">
@@ -1976,18 +2025,16 @@
         <x:v>Midazolam (IVSE)</x:v>
       </x:c>
       <x:c r="C48" s="3" t="str">
-        <x:v>Hypnovel</x:v>
-      </x:c>
-      <x:c r="D48" s="7" t="n">
-        <x:v>10</x:v>
-      </x:c>
-      <x:c r="E48" s="7" t="n">
-        <x:v>50</x:v>
-      </x:c>
+        <x:v>Midazolam 5 mg/mL — deux volumes de contenant</x:v>
+      </x:c>
+      <x:c r="D48" s="7"/>
+      <x:c r="E48" s="7"/>
       <x:c r="F48" s="6" t="str">
         <x:v>mg</x:v>
       </x:c>
-      <x:c r="G48" s="7"/>
+      <x:c r="G48" s="7" t="n">
+        <x:v>5</x:v>
+      </x:c>
       <x:c r="H48" s="9" t="n">
         <x:f>IF(AND(ISNUMBER(D48),D48&gt;0,ISNUMBER(E48),E48&gt;0),E48/D48,IF(ISNUMBER(G48),G48,""))</x:f>
         <x:v>5</x:v>
@@ -1996,7 +2043,7 @@
         <x:v>Midazolam</x:v>
       </x:c>
       <x:c r="J48" s="3" t="str">
-        <x:v>à confirmer</x:v>
+        <x:v>confirmé</x:v>
       </x:c>
       <x:c r="K48" s="3" t="str"/>
       <x:c r="L48" s="3" t="str">
@@ -2031,7 +2078,7 @@
         <x:v>Morphine</x:v>
       </x:c>
       <x:c r="J49" s="3" t="str">
-        <x:v>à confirmer</x:v>
+        <x:v>confirmé</x:v>
       </x:c>
       <x:c r="K49" s="3" t="str"/>
       <x:c r="L49" s="3" t="str">
@@ -2076,7 +2123,7 @@
         <x:v>nicardipine</x:v>
       </x:c>
       <x:c r="B51" s="3" t="str">
-        <x:v>Nicardipine (IVSE)</x:v>
+        <x:v>Nicardipine — entretien (IVSE)</x:v>
       </x:c>
       <x:c r="C51" s="3" t="str">
         <x:v>Loxen</x:v>
@@ -2096,7 +2143,7 @@
         <x:v>1</x:v>
       </x:c>
       <x:c r="I51" s="3" t="str">
-        <x:v>Nicardipine</x:v>
+        <x:v>Nicardipine — entretien</x:v>
       </x:c>
       <x:c r="J51" s="3" t="str">
         <x:v>à confirmer</x:v>
@@ -2169,7 +2216,7 @@
         <x:v>Sufentanil</x:v>
       </x:c>
       <x:c r="J53" s="3" t="str">
-        <x:v>à confirmer</x:v>
+        <x:v>confirmé</x:v>
       </x:c>
       <x:c r="K53" s="3" t="str"/>
       <x:c r="L53" s="3" t="str">
@@ -2279,36 +2326,34 @@
         <x:v>calcium-gluconate</x:v>
       </x:c>
       <x:c r="B57" s="3" t="str">
-        <x:v>Gluconate Ca2+ 10 %</x:v>
+        <x:v>Gluconate de calcium 10 %</x:v>
       </x:c>
       <x:c r="C57" s="3" t="str">
-        <x:v>Gluconate de calcium PROAMP</x:v>
+        <x:v>Gluconate de calcium 10 %</x:v>
       </x:c>
       <x:c r="D57" s="7" t="n">
         <x:v>10</x:v>
       </x:c>
-      <x:c r="E57" s="7" t="n">
-        <x:v>91</x:v>
-      </x:c>
+      <x:c r="E57" s="7"/>
       <x:c r="F57" s="6" t="str">
-        <x:v>mg</x:v>
-      </x:c>
-      <x:c r="G57" s="7"/>
+        <x:v>g</x:v>
+      </x:c>
+      <x:c r="G57" s="7" t="n">
+        <x:v>0.1</x:v>
+      </x:c>
       <x:c r="H57" s="9" t="n">
         <x:f>IF(AND(ISNUMBER(D57),D57&gt;0,ISNUMBER(E57),E57&gt;0),E57/D57,IF(ISNUMBER(G57),G57,""))</x:f>
-        <x:v>9.1</x:v>
+        <x:v>0.1</x:v>
       </x:c>
       <x:c r="I57" s="3" t="str">
-        <x:v>calcium élément (PROAMP 10 %)</x:v>
+        <x:v>concentration nominale à 10 % ; prescription en mL de solution</x:v>
       </x:c>
       <x:c r="J57" s="3" t="str">
-        <x:v>à confirmer</x:v>
-      </x:c>
-      <x:c r="K57" s="3" t="str">
-        <x:v>La dose et la dilution restent à trancher indépendamment de l’ampoule.</x:v>
-      </x:c>
+        <x:v>confirmé</x:v>
+      </x:c>
+      <x:c r="K57" s="3" t="str"/>
       <x:c r="L57" s="3" t="str">
-        <x:v>https://base-donnees-publique.medicaments.gouv.fr/medicament/68332774/extrait</x:v>
+        <x:v>Tableau Prescription / Ampoules et décisions locales de la conversation</x:v>
       </x:c>
     </x:row>
     <x:row r="58" ht="58" customHeight="1">
@@ -2316,10 +2361,10 @@
         <x:v>insuline-glucose</x:v>
       </x:c>
       <x:c r="B58" s="3" t="str">
-        <x:v>Insuline rapide + G5 %</x:v>
+        <x:v>Insuline rapide + G10 %</x:v>
       </x:c>
       <x:c r="C58" s="3" t="str">
-        <x:v>Insuline rapide — spécialité à renseigner</x:v>
+        <x:v>Insuline rapide — concentration à renseigner</x:v>
       </x:c>
       <x:c r="D58" s="7"/>
       <x:c r="E58" s="7"/>
@@ -2337,7 +2382,7 @@
         <x:v>à confirmer</x:v>
       </x:c>
       <x:c r="K58" s="3" t="str">
-        <x:v>Préciser la spécialité et sa compatibilité avec G5 %. Le second produit est une poche de 500 mL de G5 % ; mélange local : 15 UI dans 500 mL.</x:v>
+        <x:v>G10 % : 5 mL/kg (max. 250 mL). Insuline : 0,1 UI/kg (max. 10 UI). Concentration d’insuline nécessaire pour son volume de prélèvement.</x:v>
       </x:c>
       <x:c r="L58" s="3" t="str">
         <x:v>Tableau Prescription / Ampoules et décisions locales de la conversation</x:v>
@@ -2521,21 +2566,132 @@
         <x:v>Tableau Prescription / Ampoules et décisions locales de la conversation</x:v>
       </x:c>
     </x:row>
+    <x:row r="65" ht="58" customHeight="1">
+      <x:c r="A65" s="18" t="str">
+        <x:v>triphosadenine-2</x:v>
+      </x:c>
+      <x:c r="B65" s="18" t="str">
+        <x:v>Triphosadénine — 2e dose</x:v>
+      </x:c>
+      <x:c r="C65" s="18" t="str">
+        <x:v>Triphosadénine</x:v>
+      </x:c>
+      <x:c r="D65" s="21" t="n">
+        <x:v>2</x:v>
+      </x:c>
+      <x:c r="E65" s="21" t="n">
+        <x:v>20</x:v>
+      </x:c>
+      <x:c r="F65" s="19" t="str">
+        <x:v>mg</x:v>
+      </x:c>
+      <x:c r="G65" s="21"/>
+      <x:c r="H65" s="22" t="n">
+        <x:f>IF(AND(ISNUMBER(D65),D65&gt;0,ISNUMBER(E65),E65&gt;0),E65/D65,IF(ISNUMBER(G65),G65,""))</x:f>
+        <x:v>10</x:v>
+      </x:c>
+      <x:c r="I65" s="18" t="str">
+        <x:v>Triphosadénine — 2e dose</x:v>
+      </x:c>
+      <x:c r="J65" s="18" t="str">
+        <x:v>à confirmer</x:v>
+      </x:c>
+      <x:c r="K65" s="18" t="str"/>
+      <x:c r="L65" s="18" t="str">
+        <x:v>Tableau Prescription / Ampoules et décisions locales de la conversation</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="66" ht="58" customHeight="1">
+      <x:c r="A66" s="18" t="str">
+        <x:v>propofol-lisa</x:v>
+      </x:c>
+      <x:c r="B66" s="18" t="str">
+        <x:v>Propofol LISA</x:v>
+      </x:c>
+      <x:c r="C66" s="18" t="str">
+        <x:v>Propofol</x:v>
+      </x:c>
+      <x:c r="D66" s="21" t="n">
+        <x:v>20</x:v>
+      </x:c>
+      <x:c r="E66" s="21" t="n">
+        <x:v>200</x:v>
+      </x:c>
+      <x:c r="F66" s="19" t="str">
+        <x:v>mg</x:v>
+      </x:c>
+      <x:c r="G66" s="21"/>
+      <x:c r="H66" s="22" t="n">
+        <x:f>IF(AND(ISNUMBER(D66),D66&gt;0,ISNUMBER(E66),E66&gt;0),E66/D66,IF(ISNUMBER(G66),G66,""))</x:f>
+        <x:v>10</x:v>
+      </x:c>
+      <x:c r="I66" s="18" t="str">
+        <x:v>Propofol LISA</x:v>
+      </x:c>
+      <x:c r="J66" s="18" t="str">
+        <x:v>confirmé</x:v>
+      </x:c>
+      <x:c r="K66" s="18" t="str"/>
+      <x:c r="L66" s="18" t="str">
+        <x:v>Tableau Prescription / Ampoules et décisions locales de la conversation</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="67" ht="58" customHeight="1">
+      <x:c r="A67" s="18" t="str">
+        <x:v>nicardipine-charge</x:v>
+      </x:c>
+      <x:c r="B67" s="18" t="str">
+        <x:v>Nicardipine — dose de charge (IVSE)</x:v>
+      </x:c>
+      <x:c r="C67" s="18" t="str">
+        <x:v>Nicardipine</x:v>
+      </x:c>
+      <x:c r="D67" s="21" t="n">
+        <x:v>10</x:v>
+      </x:c>
+      <x:c r="E67" s="21" t="n">
+        <x:v>10</x:v>
+      </x:c>
+      <x:c r="F67" s="19" t="str">
+        <x:v>mg</x:v>
+      </x:c>
+      <x:c r="G67" s="21"/>
+      <x:c r="H67" s="22" t="n">
+        <x:f>IF(AND(ISNUMBER(D67),D67&gt;0,ISNUMBER(E67),E67&gt;0),E67/D67,IF(ISNUMBER(G67),G67,""))</x:f>
+        <x:v>1</x:v>
+      </x:c>
+      <x:c r="I67" s="18" t="str">
+        <x:v>Nicardipine — dose de charge</x:v>
+      </x:c>
+      <x:c r="J67" s="18" t="str">
+        <x:v>à confirmer</x:v>
+      </x:c>
+      <x:c r="K67" s="18" t="str"/>
+      <x:c r="L67" s="18" t="str">
+        <x:v>Tableau Prescription / Ampoules et décisions locales de la conversation</x:v>
+      </x:c>
+    </x:row>
   </x:sheetData>
   <x:conditionalFormatting sqref="J2:J64">
     <x:cfRule type="containsText" dxfId="0" priority="1" operator="containsText" text="à confirmer"/>
   </x:conditionalFormatting>
-  <x:dataValidations count="2">
+  <x:dataValidations count="4">
     <x:dataValidation type="list" sqref="J2:J64">
       <x:formula1>"confirmé,à confirmer,sans objet"</x:formula1>
     </x:dataValidation>
     <x:dataValidation type="list" sqref="F2:F64">
       <x:formula1>"g,mg,mcg,ng,mmol,UI"</x:formula1>
     </x:dataValidation>
+    <x:dataValidation type="list" sqref="F2:F67">
+      <x:formula1>"g,mg,mcg,ng,mmol,UI"</x:formula1>
+    </x:dataValidation>
+    <x:dataValidation type="list" sqref="J2:J67">
+      <x:formula1>"confirmé,à confirmer,sans objet"</x:formula1>
+    </x:dataValidation>
   </x:dataValidations>
   <x:pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <x:tableParts count="1">
-    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="Rc0165404d5804acf"/>
+    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="Rcf0ebf68c7c240a3"/>
   </x:tableParts>
 </x:worksheet>
 </file>
@@ -2553,7 +2709,7 @@
         <x:v>PediDoses — Tableau des ampoules</x:v>
       </x:c>
       <x:c r="B1" s="15" t="str">
-        <x:v>Version initiale : v0.6 — une ligne par fiche et par voie.</x:v>
+        <x:v>Version v0.9 — 66 lignes, une par fiche et par voie.</x:v>
       </x:c>
     </x:row>
     <x:row r="2" ht="80" customHeight="1">
@@ -2625,7 +2781,7 @@
         <x:v>9. Sulfate de magnésium</x:v>
       </x:c>
       <x:c r="B10" s="3" t="str">
-        <x:v>Volume : 10 mL. Quantité totale laissée vide : la saisie « 0,15 g » doit être précisée (par mL ou par ampoule). Une solution à 15 % correspond à 1,5 g/10 mL. Dans l’application, aucun volume n’est calculé avant confirmation.</x:v>
+        <x:v>Sulfate de magnésium 15 % confirmé : 1,5 g dans 10 mL (150 mg/mL). Le volume à prélever est calculé ; la dilution finale reste à préciser.</x:v>
       </x:c>
     </x:row>
     <x:row r="11" ht="80" customHeight="1">
@@ -2633,7 +2789,7 @@
         <x:v>10. Insuline et glucose</x:v>
       </x:c>
       <x:c r="B11" s="3" t="str">
-        <x:v>La ligne décrit l’insuline rapide à identifier. Le second produit est une poche de G5 % de 500 mL. Le mélange local demeure 15 UI dans 500 mL ; préciser la compatibilité de la spécialité avec G5 %.</x:v>
+        <x:v>Insuline rapide : 0,1 UI/kg, maximum 10 UI. G10 % : 5 mL/kg, maximum 250 mL. Administration sur 30 min. Les plafonds sont indépendants ; la concentration de l’insuline reste à renseigner pour calculer son prélèvement.</x:v>
       </x:c>
     </x:row>
     <x:row r="12" ht="80" customHeight="1">
@@ -2641,7 +2797,7 @@
         <x:v>11. Triphosadénine</x:v>
       </x:c>
       <x:c r="B12" s="3" t="str">
-        <x:v>Posologie, préparation et administration laissées en suspens à la demande du prescripteur, faute d’informations. Aucun calcul automatique.</x:v>
+        <x:v>1re dose : 1 mg/kg, maximum 10 mg. 2e dose : 2 mg/kg, maximum 20 mg. Modalités IV à préciser.</x:v>
       </x:c>
     </x:row>
     <x:row r="13" ht="80" customHeight="1">

</xml_diff>